<commit_message>
Spark: RLUSD/USDS V4 pool (S66) + S61 is not an SDE + LP-NFT detector + CoF base fix (#184)
Co-authored-by: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/spark/2026-08/spark_settlement_august_2026.xlsx
+++ b/settlements/spark/2026-08/spark_settlement_august_2026.xlsx
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>6366152.050719894</v>
+        <v>6365737.750085554</v>
       </c>
     </row>
     <row r="5">
@@ -517,7 +517,7 @@
     <row r="7">
       <c r="A7" t="inlineStr"/>
       <c r="B7" s="4" t="n">
-        <v>7205832.009352266</v>
+        <v>7205417.708717926</v>
       </c>
     </row>
     <row r="9">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>6084935.362245966</v>
+        <v>6267981.96185068</v>
       </c>
     </row>
     <row r="11">
@@ -549,13 +549,13 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>-7778.867166258307</v>
+        <v>-7825.937104839475</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
       <c r="B12" s="4" t="n">
-        <v>6077156.495079707</v>
+        <v>6260156.024745842</v>
       </c>
     </row>
     <row r="14">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>6084935.362245966</v>
+        <v>6267981.96185068</v>
       </c>
     </row>
     <row r="16">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>-2078993.144321223</v>
+        <v>-1895946.544716508</v>
       </c>
     </row>
     <row r="17">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>6366152.050719894</v>
+        <v>6365737.750085554</v>
       </c>
     </row>
     <row r="23">
@@ -635,13 +635,13 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>-6084935.362245966</v>
+        <v>-6267981.96185068</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" s="4" t="n">
-        <v>115561.8154067152</v>
+        <v>-67899.08483233953</v>
       </c>
     </row>
     <row r="26">
@@ -676,7 +676,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-09-01T17:50:05+00:00</t>
+          <t>2026-09-02T13:24:59+00:00</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S67"/>
+  <dimension ref="A1:S68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -873,13 +873,13 @@
         <v>1</v>
       </c>
       <c r="N2" s="6" t="n">
-        <v>1801452.451759816</v>
+        <v>1805407.625659391</v>
       </c>
       <c r="O2" s="6" t="n">
-        <v>1801452.451759816</v>
+        <v>1805407.625659391</v>
       </c>
       <c r="P2" s="6" t="n">
-        <v>-632993.1092491396</v>
+        <v>-636948.2831487146</v>
       </c>
       <c r="Q2" s="6" t="n">
         <v>0</v>
@@ -938,13 +938,13 @@
         <v>1</v>
       </c>
       <c r="N3" s="6" t="n">
-        <v>1242788.075922378</v>
+        <v>1245516.675811756</v>
       </c>
       <c r="O3" s="6" t="n">
-        <v>1242788.075922378</v>
+        <v>1245516.675811756</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>59902.44485108774</v>
+        <v>57173.8449617099</v>
       </c>
       <c r="Q3" s="6" t="n">
         <v>291031640.1762941</v>
@@ -1007,13 +1007,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="6" t="n">
-        <v>994771.4678228415</v>
+        <v>996955.5355409383</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>994771.4678228415</v>
+        <v>996955.5355409383</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>157078.6498921585</v>
+        <v>154894.5821740618</v>
       </c>
       <c r="Q4" s="6" t="n">
         <v>0</v>
@@ -1072,13 +1072,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>636040.9858473208</v>
+        <v>637437.4438575369</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>636040.9858473208</v>
+        <v>637437.4438575369</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>606349.2241526782</v>
+        <v>604952.7661424621</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>0</v>
@@ -1137,13 +1137,13 @@
         <v>1</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>497135.3333348593</v>
+        <v>498226.8174276211</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>497135.3333348593</v>
+        <v>498226.8174276211</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>37692.81041203155</v>
+        <v>36601.32631926976</v>
       </c>
       <c r="Q6" s="6" t="n">
         <v>106660153.3978665</v>
@@ -1206,13 +1206,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>270329.3260452586</v>
+        <v>270922.8468421131</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>270329.3260452586</v>
+        <v>270922.8468421131</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>-229201.7342722586</v>
+        <v>-229795.2550691131</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>0</v>
@@ -1271,13 +1271,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>267298.615192602</v>
+        <v>267885.4819207077</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>267298.615192602</v>
+        <v>267885.4819207077</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>21924.30339665968</v>
+        <v>21337.43666855395</v>
       </c>
       <c r="Q8" s="6" t="n">
         <v>0</v>
@@ -1336,13 +1336,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>251206.0850793583</v>
+        <v>251757.6198979152</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>235421.577610291</v>
+        <v>235973.1124288479</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>25259.74847325789</v>
+        <v>24708.21365470095</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>0</v>
@@ -1355,12 +1355,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>S18</t>
+          <t>S61</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Arkis Spark Prime USDC 1 (ERC-4626)</t>
+          <t>Spark.fi PYUSD Reserve Uniswap V4 (PYUSD/USDS)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1370,44 +1370,44 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E10" s="6" t="n">
-        <v>20219164.29469907</v>
+        <v>100118990.9295999</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>20321999.31292716</v>
+        <v>100118954.1795337</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>102835.0182280904</v>
+        <v>-36.75006615869079</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>102835.0182280904</v>
+        <v>47.06993858116784</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>102835.0182280904</v>
+        <v>47.06993858116784</v>
       </c>
       <c r="K10" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>20219164.29469907</v>
+        <v>61436481.21524471</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>54658.93262954819</v>
+        <v>166447.2972992444</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>54658.93262954819</v>
+        <v>166447.2972992444</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>48176.08559854225</v>
+        <v>-166400.2273606633</v>
       </c>
       <c r="Q10" s="6" t="n">
         <v>0</v>
@@ -1415,17 +1415,21 @@
       <c r="R10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>(avg excl. idle AMM USDS)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>S65</t>
+          <t>S18</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Spark Blue Chip USDT Vault (Morpho — 2026-06 redeployment)</t>
+          <t>Arkis Spark Prime USDC 1 (ERC-4626)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1439,40 +1443,40 @@
         </is>
       </c>
       <c r="E11" s="6" t="n">
-        <v>60823719.84933824</v>
+        <v>20219164.29469907</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>32509163.72156616</v>
+        <v>20321999.31292716</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>-28314556.12777209</v>
+        <v>102835.0182280904</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>28244.9115647759</v>
+        <v>102835.0182280904</v>
       </c>
       <c r="I11" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>28244.9115647759</v>
+        <v>102835.0182280904</v>
       </c>
       <c r="K11" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>11240574.91722324</v>
+        <v>20219164.29469907</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>30386.90512441076</v>
+        <v>54778.9388964379</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>30386.90512441076</v>
+        <v>54778.9388964379</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>-2141.993559634862</v>
+        <v>48056.07933165254</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>0</v>
@@ -1485,12 +1489,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S65</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Spark USDC (SparkLend spToken)</t>
+          <t>Spark Blue Chip USDT Vault (Morpho — 2026-06 redeployment)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1500,44 +1504,44 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>11026528.088879</v>
+        <v>60823719.84933824</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>6825075.305007</v>
+        <v>32509163.72156616</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>-4201452.783872</v>
+        <v>-28314556.12777209</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>32569.911561</v>
+        <v>28244.9115647759</v>
       </c>
       <c r="I12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>32569.911561</v>
+        <v>28244.9115647759</v>
       </c>
       <c r="K12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>10889946.71160697</v>
+        <v>11240574.91722324</v>
       </c>
       <c r="M12" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>29439.04381869775</v>
+        <v>30453.62100909566</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>29439.04381869775</v>
+        <v>30453.62100909566</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>3130.867742302249</v>
+        <v>-2208.709444319758</v>
       </c>
       <c r="Q12" s="6" t="n">
         <v>0</v>
@@ -1550,12 +1554,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>S64</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RLUSD raw (ALM idle — $251.7M as of 2026-08)</t>
+          <t>Spark USDC (SparkLend spToken)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1565,44 +1569,44 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E13" s="6" t="n">
-        <v>0</v>
+        <v>11026528.088879</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>251703857.665157</v>
+        <v>6825075.305007</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>251703857.665157</v>
+        <v>-4201452.783872</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>0</v>
+        <v>32569.911561</v>
       </c>
       <c r="I13" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>0</v>
+        <v>32569.911561</v>
       </c>
       <c r="K13" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>8119479.279521191</v>
+        <v>10889946.71160697</v>
       </c>
       <c r="M13" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N13" s="6" t="n">
-        <v>21949.57538589834</v>
+        <v>29503.67862913997</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>21949.57538589834</v>
+        <v>29503.67862913997</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>-21949.57538589834</v>
+        <v>3066.232931860034</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>0</v>
@@ -1615,12 +1619,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S64</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Spark Blue Chip USDC Vault (Morpho)</t>
+          <t>RLUSD raw (ALM idle — $251.7M as of 2026-08)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1630,44 +1634,44 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>772030.6797926712</v>
+        <v>0</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>11021603.25234972</v>
+        <v>251703857.665157</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>10249572.57255705</v>
+        <v>251703857.665157</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>13511.81533200658</v>
+        <v>0</v>
       </c>
       <c r="I14" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>13511.81533200658</v>
+        <v>0</v>
       </c>
       <c r="K14" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>4227772.364670921</v>
+        <v>8119479.279521191</v>
       </c>
       <c r="M14" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N14" s="6" t="n">
-        <v>11429.0344291924</v>
+        <v>21997.76671483863</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>11429.0344291924</v>
+        <v>21997.76671483863</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>2082.780902814179</v>
+        <v>-21997.76671483863</v>
       </c>
       <c r="Q14" s="6" t="n">
         <v>0</v>
@@ -1680,96 +1684,92 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SPREAD</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>30bps sUSDS spread (Curve LP + PSM3) — Sky Revenue reduction</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+          <t>Spark Blue Chip USDC Vault (Morpho)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="E15" s="6" t="n">
-        <v>0</v>
+        <v>772030.6797926712</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>0</v>
+        <v>11021603.25234972</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>0</v>
+        <v>10249572.57255705</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>0</v>
+        <v>13511.81533200658</v>
       </c>
       <c r="I15" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>0</v>
+        <v>13511.81533200658</v>
       </c>
       <c r="K15" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>0</v>
+        <v>4227772.364670921</v>
       </c>
       <c r="M15" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>0</v>
+        <v>11454.12741381574</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>-8190.469335843211</v>
+        <v>11454.12741381574</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>0</v>
+        <v>2057.687918190839</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>0</v>
       </c>
       <c r="R15" s="6" t="n">
-        <v>8190.469335843211</v>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>sky-revenue reduction (no CoF; computed outside venue loop)</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="S15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>S62</t>
+          <t>SPREAD</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Spark.fi USDT Reserve Uniswap V4 (USDT/USDS)</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>ethereum</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
+          <t>30bps sUSDS spread (Curve LP + PSM3) — Sky Revenue reduction</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" s="6" t="n">
-        <v>50000939.1994665</v>
+        <v>0</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>50000607.68881255</v>
+        <v>0</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>-331.5106539449819</v>
+        <v>0</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>-7825.941992720887</v>
+        <v>0</v>
       </c>
       <c r="I16" s="6" t="n">
         <v>0</v>
@@ -1778,10 +1778,10 @@
         <v>0</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>-7825.941992720887</v>
+        <v>0</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>50003821.81122544</v>
+        <v>0</v>
       </c>
       <c r="M16" s="7" t="n">
         <v>0</v>
@@ -1790,32 +1790,32 @@
         <v>0</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>-7825.941992720887</v>
+        <v>-8190.469335843211</v>
       </c>
       <c r="P16" s="6" t="n">
         <v>0</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>50003821.81122544</v>
+        <v>0</v>
       </c>
       <c r="R16" s="6" t="n">
-        <v>0</v>
+        <v>8190.469335843211</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>SDE (fixed)</t>
+          <t>sky-revenue reduction (no CoF; computed outside venue loop)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>S61</t>
+          <t>S62</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Spark.fi PYUSD Reserve Uniswap V4 (PYUSD/USDS)</t>
+          <t>Spark.fi USDT Reserve Uniswap V4 (USDT/USDS)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1829,16 +1829,16 @@
         </is>
       </c>
       <c r="E17" s="6" t="n">
-        <v>100118990.9295999</v>
+        <v>50000939.1994665</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>100118954.1795337</v>
+        <v>50000607.68881255</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>-36.75006615869079</v>
+        <v>-331.5106539449819</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>47.06993858116784</v>
+        <v>-7825.941992720887</v>
       </c>
       <c r="I17" s="6" t="n">
         <v>0</v>
@@ -1847,10 +1847,10 @@
         <v>0</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>47.06993858116784</v>
+        <v>-7825.941992720887</v>
       </c>
       <c r="L17" s="6" t="n">
-        <v>100118885.4440565</v>
+        <v>37183169.59569638</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>0</v>
@@ -1859,32 +1859,32 @@
         <v>0</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>47.06993858116784</v>
+        <v>-7825.941992720887</v>
       </c>
       <c r="P17" s="6" t="n">
         <v>0</v>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>100118885.4440565</v>
+        <v>37183169.59569638</v>
       </c>
       <c r="R17" s="6" t="n">
         <v>0</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>SDE (fixed)</t>
+          <t>SDE (fixed) (avg excl. idle AMM USDS)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>S27</t>
+          <t>S66</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>USDT raw (ALM idle — $442M as of 2026-04)</t>
+          <t>Spark.fi RLUSD Reserve Uniswap V4 (RLUSD/USDS)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1894,44 +1894,44 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>6730.269529</v>
+        <v>0</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>0</v>
+        <v>19999704.07519871</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-6730.269529</v>
+        <v>19999704.07519871</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>0</v>
+        <v>-461.370572920806</v>
       </c>
       <c r="I18" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>0</v>
+        <v>-461.370572920806</v>
       </c>
       <c r="K18" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="6" t="n">
-        <v>6513.164060322581</v>
+        <v>1176300.265828546</v>
       </c>
       <c r="M18" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>17.60718644893255</v>
+        <v>3186.901270819541</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>17.60718644893255</v>
+        <v>3186.901270819541</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>-17.60718644893255</v>
+        <v>-3648.271843740347</v>
       </c>
       <c r="Q18" s="6" t="n">
         <v>0</v>
@@ -1939,22 +1939,26 @@
       <c r="R18" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S18" t="inlineStr"/>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>(avg excl. idle AMM USDS)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>S39</t>
+          <t>S27</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>USDC raw (Base — ALM idle)</t>
+          <t>USDT raw (ALM idle — $442M as of 2026-04)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1963,13 +1967,13 @@
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>1326.975817</v>
+        <v>6730.269529</v>
       </c>
       <c r="F19" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>-1326.975817</v>
+        <v>-6730.269529</v>
       </c>
       <c r="H19" s="6" t="n">
         <v>0</v>
@@ -1984,19 +1988,19 @@
         <v>0</v>
       </c>
       <c r="L19" s="6" t="n">
-        <v>1284.170145483871</v>
+        <v>6513.164060322581</v>
       </c>
       <c r="M19" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>3.471526737892046</v>
+        <v>17.64584385796921</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>3.471526737892046</v>
+        <v>17.64584385796921</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>-3.471526737892046</v>
+        <v>-17.64584385796921</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>0</v>
@@ -2009,59 +2013,59 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S39</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Spark DAI Vault (Morpho)</t>
+          <t>USDC raw (Base — ALM idle)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>725.7224774532416</v>
+        <v>1326.975817</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>907.5387997189844</v>
+        <v>0</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>181.8163222657428</v>
+        <v>-1326.975817</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>139.2163980605023</v>
+        <v>0</v>
       </c>
       <c r="I20" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>139.2163980605023</v>
+        <v>0</v>
       </c>
       <c r="K20" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>750.4579173143489</v>
+        <v>1284.170145483871</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>2.028730176278858</v>
+        <v>3.479148638726549</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>2.028730176278858</v>
+        <v>3.479148638726549</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>137.1876678842234</v>
+        <v>-3.479148638726549</v>
       </c>
       <c r="Q20" s="6" t="n">
         <v>0</v>
@@ -2074,17 +2078,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>S36</t>
+          <t>S12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Fluid Savings USDS (fsUSDS, Base)</t>
+          <t>Spark DAI Vault (Morpho)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2093,40 +2097,40 @@
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>283.8972488542868</v>
+        <v>725.7224774532416</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>283.8972488542868</v>
+        <v>907.5387997189844</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>0</v>
+        <v>181.8163222657428</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>0</v>
+        <v>139.2163980605023</v>
       </c>
       <c r="I21" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>0</v>
+        <v>139.2163980605023</v>
       </c>
       <c r="K21" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="6" t="n">
-        <v>283.8972488542868</v>
+        <v>750.4579173143489</v>
       </c>
       <c r="M21" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N21" s="6" t="n">
-        <v>0.7674659730080347</v>
+        <v>2.033184349151786</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>0.7674659730080347</v>
+        <v>2.033184349151786</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>-0.7674659730080347</v>
+        <v>137.1832137113505</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>0</v>
@@ -2139,17 +2143,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>S16</t>
+          <t>S36</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ethena Staked USDe (sUSDe)</t>
+          <t>Fluid Savings USDS (fsUSDS, Base)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2158,40 +2162,40 @@
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>100.4548689419015</v>
+        <v>283.8972488542868</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>100.8102461380194</v>
+        <v>283.8972488542868</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>0.3553771961178877</v>
+        <v>0</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0.3553771961178877</v>
+        <v>0</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.3553771961178877</v>
+        <v>0</v>
       </c>
       <c r="K22" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>100.4548689419015</v>
+        <v>283.8972488542868</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N22" s="6" t="n">
-        <v>0.271561961403371</v>
+        <v>0.769150980781783</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>0.271561961403371</v>
+        <v>0.769150980781783</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>0.08381523471451675</v>
+        <v>-0.769150980781783</v>
       </c>
       <c r="Q22" s="6" t="n">
         <v>0</v>
@@ -2204,59 +2208,59 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>S49</t>
+          <t>S16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>USDC raw (Optimism — ALM idle)</t>
+          <t>Ethena Staked USDe (sUSDe)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>optimism</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0</v>
+        <v>100.4548689419015</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>3039.891609</v>
+        <v>100.8102461380194</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>3039.891609</v>
+        <v>0.3553771961178877</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>0</v>
+        <v>0.3553771961178877</v>
       </c>
       <c r="I23" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>0</v>
+        <v>0.3553771961178877</v>
       </c>
       <c r="K23" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>98.06101964516129</v>
+        <v>100.4548689419015</v>
       </c>
       <c r="M23" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N23" s="6" t="n">
-        <v>0.2650906134520554</v>
+        <v>0.2721581885093435</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>0.2650906134520554</v>
+        <v>0.2721581885093435</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>-0.2650906134520554</v>
+        <v>0.08321900760854414</v>
       </c>
       <c r="Q23" s="6" t="n">
         <v>0</v>
@@ -2269,59 +2273,59 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>S13</t>
+          <t>S49</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Spark USDS Vault (Morpho)</t>
+          <t>USDC raw (Optimism — ALM idle)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>optimism</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>21.94239521151591</v>
+        <v>0</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>22.16728989737678</v>
+        <v>3039.891609</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>0.2248946858608627</v>
+        <v>3039.891609</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0.2248946858608627</v>
+        <v>0</v>
       </c>
       <c r="I24" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J24" s="6" t="n">
-        <v>0.2248946858608627</v>
+        <v>0</v>
       </c>
       <c r="K24" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>21.94239521151591</v>
+        <v>98.06101964516129</v>
       </c>
       <c r="M24" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>0.05931738246528844</v>
+        <v>0.2656726324081059</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>0.05931738246528844</v>
+        <v>0.2656726324081059</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>0.1655773033955742</v>
+        <v>-0.2656726324081059</v>
       </c>
       <c r="Q24" s="6" t="n">
         <v>0</v>
@@ -2334,12 +2338,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>S9</t>
+          <t>S13</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Aave Ethereum USDT (aToken)</t>
+          <t>Spark USDS Vault (Morpho)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2349,44 +2353,44 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>5.938459</v>
+        <v>21.94239521151591</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>5.953731</v>
+        <v>22.16728989737678</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>0.015272</v>
+        <v>0.2248946858608627</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>0.015272</v>
+        <v>0.2248946858608627</v>
       </c>
       <c r="I25" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>0.015272</v>
+        <v>0.2248946858608627</v>
       </c>
       <c r="K25" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>5.938459</v>
+        <v>21.94239521151591</v>
       </c>
       <c r="M25" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>0.01605357301980245</v>
+        <v>0.05944761657870544</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>0.01605357301980245</v>
+        <v>0.05944761657870544</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>-0.0007815730198024501</v>
+        <v>0.1654470692821573</v>
       </c>
       <c r="Q25" s="6" t="n">
         <v>0</v>
@@ -2399,12 +2403,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>S25</t>
+          <t>S9</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Spark.fi PYUSD Reserve Curve (PYUSD/USDS)</t>
+          <t>Aave Ethereum USDT (aToken)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2414,44 +2418,44 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>3.882540733930369</v>
+        <v>5.938459</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>3.882840172509015</v>
+        <v>5.953731</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>0.0002994385786456635</v>
+        <v>0.015272</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>0.0002994385786456635</v>
+        <v>0.015272</v>
       </c>
       <c r="I26" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J26" s="6" t="n">
-        <v>0.0002994385786456635</v>
+        <v>0.015272</v>
       </c>
       <c r="K26" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>3.882540733930369</v>
+        <v>5.938459</v>
       </c>
       <c r="M26" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>0.01049576180866258</v>
+        <v>0.01608881939721353</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>0.01049576180866258</v>
+        <v>0.01608881939721353</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>-0.01019632323001692</v>
+        <v>-0.0008168193972135317</v>
       </c>
       <c r="Q26" s="6" t="n">
         <v>0</v>
@@ -2464,12 +2468,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>S24</t>
+          <t>S25</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Spark.fi USDT Reserve Curve (sUSDS/USDT)</t>
+          <t>Spark.fi PYUSD Reserve Curve (PYUSD/USDS)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2483,62 +2487,58 @@
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>0.8244687442276728</v>
+        <v>3.882540733930369</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>0.8298484399352527</v>
+        <v>3.882840172509015</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>0.005379695707579953</v>
+        <v>0.0002994385786456635</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>0.004887881412778414</v>
+        <v>0.0002994385786456635</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>0.0004918142948015394</v>
+        <v>0</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>0.0004918142948015394</v>
+        <v>0.0002994385786456635</v>
       </c>
       <c r="K27" s="6" t="n">
-        <v>0.004887881412778414</v>
+        <v>0</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>0.8244687442276728</v>
+        <v>3.882540733930369</v>
       </c>
       <c r="M27" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>0</v>
+        <v>0.01051880574919025</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>0.004887881412778414</v>
+        <v>0.01051880574919025</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.0004918142948015394</v>
+        <v>-0.01021936717054459</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>0.8244687442276728</v>
+        <v>0</v>
       </c>
       <c r="R27" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>SDE (fixed)</t>
-        </is>
-      </c>
+      <c r="S27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S24</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Spark Blue Chip USDT Vault (Morpho — pre-2026-06 deployment)</t>
+          <t>Spark.fi USDT Reserve Curve (sUSDS/USDT)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2548,62 +2548,66 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>1.75807157545523</v>
+        <v>0.8244687442276728</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>1.762330143465235</v>
+        <v>0.8298484399352527</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>0.004258568010004908</v>
+        <v>0.005379695707579953</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>0.004258568010004908</v>
+        <v>0.004887881412778414</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>0</v>
+        <v>0.0004918142948015394</v>
       </c>
       <c r="J28" s="6" t="n">
-        <v>0.004258568010004908</v>
+        <v>0.0004918142948015394</v>
       </c>
       <c r="K28" s="6" t="n">
-        <v>0</v>
+        <v>0.004887881412778414</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>1.75807157545523</v>
+        <v>0.8244687442276728</v>
       </c>
       <c r="M28" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>0.004752635390866498</v>
+        <v>0</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>0.004752635390866498</v>
+        <v>0.004887881412778414</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>-0.0004940673808615894</v>
+        <v>0.0004918142948015394</v>
       </c>
       <c r="Q28" s="6" t="n">
-        <v>0</v>
+        <v>0.8244687442276728</v>
       </c>
       <c r="R28" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S28" t="inlineStr"/>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>SDE (fixed)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>S23</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Anchorage tri-party loan escrow (USDC pass-through, ~$0 balance)</t>
+          <t>Spark Blue Chip USDT Vault (Morpho — pre-2026-06 deployment)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2613,44 +2617,44 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>1.359103</v>
+        <v>1.75807157545523</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>40137.360529</v>
+        <v>1.762330143465235</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>40136.001426</v>
+        <v>0.004258568010004908</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>40136.001426</v>
+        <v>0.004258568010004908</v>
       </c>
       <c r="I29" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J29" s="6" t="n">
-        <v>40136.001426</v>
+        <v>0.004258568010004908</v>
       </c>
       <c r="K29" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>1.359103</v>
+        <v>1.75807157545523</v>
       </c>
       <c r="M29" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>0.003674094449744045</v>
+        <v>0.004763070026226309</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>0.003674094449744045</v>
+        <v>0.004763070026226309</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>40135.99775190555</v>
+        <v>-0.0005045020162214007</v>
       </c>
       <c r="Q29" s="6" t="n">
         <v>0</v>
@@ -2663,59 +2667,59 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>S54</t>
+          <t>S23</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Aave Avalanche USDC (aAvaUSDC)</t>
+          <t>Anchorage tri-party loan escrow (USDC pass-through, ~$0 balance)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>avalanche_c</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>0.156077</v>
+        <v>1.359103</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>0.156574</v>
+        <v>40137.360529</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>0.000497</v>
+        <v>40136.001426</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>0.000497</v>
+        <v>40136.001426</v>
       </c>
       <c r="I30" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J30" s="6" t="n">
-        <v>0.000497</v>
+        <v>40136.001426</v>
       </c>
       <c r="K30" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>0.156077</v>
+        <v>1.359103</v>
       </c>
       <c r="M30" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N30" s="6" t="n">
-        <v>0.0004219265496674654</v>
+        <v>0.003682161097552598</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>0.0004219265496674654</v>
+        <v>0.003682161097552598</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>7.507345033253459e-05</v>
+        <v>40135.9977438389</v>
       </c>
       <c r="Q30" s="6" t="n">
         <v>0</v>
@@ -2728,59 +2732,59 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>S45</t>
+          <t>S54</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>USDC raw (Arbitrum — ALM idle)</t>
+          <t>Aave Avalanche USDC (aAvaUSDC)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>arbitrum</t>
+          <t>avalanche_c</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>0</v>
+        <v>0.156077</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>2.08</v>
+        <v>0.156574</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>2.08</v>
+        <v>0.000497</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>0</v>
+        <v>0.000497</v>
       </c>
       <c r="I31" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>0</v>
+        <v>0.000497</v>
       </c>
       <c r="K31" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L31" s="6" t="n">
-        <v>0.06709677419354838</v>
+        <v>0.156077</v>
       </c>
       <c r="M31" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N31" s="6" t="n">
-        <v>0.0001813842553950993</v>
+        <v>0.0004228529093252806</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>0.0001813842553950993</v>
+        <v>0.0004228529093252806</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>-0.0001813842553950993</v>
+        <v>7.414709067471942e-05</v>
       </c>
       <c r="Q31" s="6" t="n">
         <v>0</v>
@@ -2793,59 +2797,59 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>S8</t>
+          <t>S45</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Aave Ethereum USDC (aToken)</t>
+          <t>USDC raw (Arbitrum — ALM idle)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>arbitrum</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>0.058302</v>
+        <v>0</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>0.058479</v>
+        <v>2.08</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>0.000177</v>
+        <v>2.08</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>0.000177</v>
+        <v>0</v>
       </c>
       <c r="I32" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J32" s="6" t="n">
-        <v>0.000177</v>
+        <v>0</v>
       </c>
       <c r="K32" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L32" s="6" t="n">
-        <v>0.058302</v>
+        <v>0.06709677419354838</v>
       </c>
       <c r="M32" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N32" s="6" t="n">
-        <v>0.0001576091397112487</v>
+        <v>0.0001817824930904832</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>0.0001576091397112487</v>
+        <v>0.0001817824930904832</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>1.939086028875127e-05</v>
+        <v>-0.0001817824930904832</v>
       </c>
       <c r="Q32" s="6" t="n">
         <v>0</v>
@@ -2858,17 +2862,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>S41</t>
+          <t>S8</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Aave Arbitrum USDCn (aArbUSDCn)</t>
+          <t>Aave Ethereum USDC (aToken)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>arbitrum</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2877,40 +2881,40 @@
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>0.006389</v>
+        <v>0.058302</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>0.006402</v>
+        <v>0.058479</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>1.3e-05</v>
+        <v>0.000177</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>1.3e-05</v>
+        <v>0.000177</v>
       </c>
       <c r="I33" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J33" s="6" t="n">
-        <v>1.3e-05</v>
+        <v>0.000177</v>
       </c>
       <c r="K33" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L33" s="6" t="n">
-        <v>0.006389</v>
+        <v>0.058302</v>
       </c>
       <c r="M33" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N33" s="6" t="n">
-        <v>1.727153088427787e-05</v>
+        <v>0.0001579551780177894</v>
       </c>
       <c r="O33" s="6" t="n">
-        <v>1.727153088427787e-05</v>
+        <v>0.0001579551780177894</v>
       </c>
       <c r="P33" s="6" t="n">
-        <v>-4.271530884277866e-06</v>
+        <v>1.904482198221065e-05</v>
       </c>
       <c r="Q33" s="6" t="n">
         <v>0</v>
@@ -2923,17 +2927,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>S7</t>
+          <t>S41</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Aave Ethereum USDS (aToken)</t>
+          <t>Aave Arbitrum USDCn (aArbUSDCn)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>arbitrum</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2942,40 +2946,40 @@
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>0.005748588443741238</v>
+        <v>0.006389</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>0.005749186661712982</v>
+        <v>0.006402</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>5.98217971744e-07</v>
+        <v>1.3e-05</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>5.98217971744e-07</v>
+        <v>1.3e-05</v>
       </c>
       <c r="I34" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J34" s="6" t="n">
-        <v>5.98217971744e-07</v>
+        <v>1.3e-05</v>
       </c>
       <c r="K34" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L34" s="6" t="n">
-        <v>0.005748588443741238</v>
+        <v>0.006389</v>
       </c>
       <c r="M34" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>1.554029157099384e-05</v>
+        <v>1.730945134567693e-05</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>1.554029157099384e-05</v>
+        <v>1.730945134567693e-05</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>-1.494207359924984e-05</v>
+        <v>-4.309451345676926e-06</v>
       </c>
       <c r="Q34" s="6" t="n">
         <v>0</v>
@@ -2988,17 +2992,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>S35</t>
+          <t>S7</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Aave Base USDC (aBasUSDC)</t>
+          <t>Aave Ethereum USDS (aToken)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3007,40 +3011,40 @@
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>0.001714</v>
+        <v>0.005748588443741238</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>0.001719</v>
+        <v>0.005749186661712982</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>5e-06</v>
+        <v>5.98217971744e-07</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>5e-06</v>
+        <v>5.98217971744e-07</v>
       </c>
       <c r="I35" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>5e-06</v>
+        <v>5.98217971744e-07</v>
       </c>
       <c r="K35" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L35" s="6" t="n">
-        <v>0.001714</v>
+        <v>0.005748588443741238</v>
       </c>
       <c r="M35" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N35" s="6" t="n">
-        <v>4.633495685655386e-06</v>
+        <v>1.557441101475342e-05</v>
       </c>
       <c r="O35" s="6" t="n">
-        <v>4.633495685655386e-06</v>
+        <v>1.557441101475342e-05</v>
       </c>
       <c r="P35" s="6" t="n">
-        <v>3.665043143446137e-07</v>
+        <v>-1.497619304300942e-05</v>
       </c>
       <c r="Q35" s="6" t="n">
         <v>0</v>
@@ -3053,59 +3057,59 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>S17</t>
+          <t>S35</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Fluid Savings USDS (fsUSDS)</t>
+          <t>Aave Base USDC (aBasUSDC)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>0.001240144670509943</v>
+        <v>0.001714</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>0.001240144670509943</v>
+        <v>0.001719</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>0</v>
+        <v>5e-06</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>0</v>
+        <v>5e-06</v>
       </c>
       <c r="I36" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J36" s="6" t="n">
-        <v>0</v>
+        <v>5e-06</v>
       </c>
       <c r="K36" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L36" s="6" t="n">
-        <v>0.001240144670509943</v>
+        <v>0.001714</v>
       </c>
       <c r="M36" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>3.352511657174062e-06</v>
+        <v>4.643668744168141e-06</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>3.352511657174062e-06</v>
+        <v>4.643668744168141e-06</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>-3.352511657174062e-06</v>
+        <v>3.563312558318592e-07</v>
       </c>
       <c r="Q36" s="6" t="n">
         <v>0</v>
@@ -3118,12 +3122,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>S17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Aave Ethereum Lido USDS (aToken)</t>
+          <t>Fluid Savings USDS (fsUSDS)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3133,44 +3137,44 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>0.000522446400962938</v>
+        <v>0.001240144670509943</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>0.000522802561158111</v>
+        <v>0.001240144670509943</v>
       </c>
       <c r="G37" s="6" t="n">
-        <v>3.56160195173e-07</v>
+        <v>0</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>3.56160195173e-07</v>
+        <v>0</v>
       </c>
       <c r="I37" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J37" s="6" t="n">
-        <v>3.56160195173e-07</v>
+        <v>0</v>
       </c>
       <c r="K37" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L37" s="6" t="n">
-        <v>0.000522446400962938</v>
+        <v>0.001240144670509943</v>
       </c>
       <c r="M37" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>1.412341391393207e-06</v>
+        <v>3.359872254780467e-06</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>1.412341391393207e-06</v>
+        <v>3.359872254780467e-06</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>-1.056181196220207e-06</v>
+        <v>-3.359872254780467e-06</v>
       </c>
       <c r="Q37" s="6" t="n">
         <v>0</v>
@@ -3183,12 +3187,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>S30</t>
+          <t>S6</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>USDe raw (ALM idle)</t>
+          <t>Aave Ethereum Lido USDS (aToken)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -3198,44 +3202,44 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>7.4896275897803e-05</v>
+        <v>0.000522446400962938</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>7.4896275897803e-05</v>
+        <v>0.000522802561158111</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>0</v>
+        <v>3.56160195173e-07</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>0</v>
+        <v>3.56160195173e-07</v>
       </c>
       <c r="I38" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J38" s="6" t="n">
-        <v>0</v>
+        <v>3.56160195173e-07</v>
       </c>
       <c r="K38" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>7.4896275897803e-05</v>
+        <v>0.000522446400962938</v>
       </c>
       <c r="M38" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>2.024688280304117e-07</v>
+        <v>1.415442253590858e-06</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>2.024688280304117e-07</v>
+        <v>1.415442253590858e-06</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>-2.024688280304117e-07</v>
+        <v>-1.059282058417858e-06</v>
       </c>
       <c r="Q38" s="6" t="n">
         <v>0</v>
@@ -3248,12 +3252,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>S14</t>
+          <t>S30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Maple syrupUSDC (ERC-4626)</t>
+          <t>USDe raw (ALM idle)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -3263,44 +3267,44 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E39" s="6" t="n">
-        <v>1.176169e-06</v>
+        <v>7.4896275897803e-05</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>1.18094e-06</v>
+        <v>7.4896275897803e-05</v>
       </c>
       <c r="G39" s="6" t="n">
-        <v>4.771e-09</v>
+        <v>0</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>4.771e-09</v>
+        <v>0</v>
       </c>
       <c r="I39" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J39" s="6" t="n">
-        <v>4.771e-09</v>
+        <v>0</v>
       </c>
       <c r="K39" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L39" s="6" t="n">
-        <v>1.176169e-06</v>
+        <v>7.4896275897803e-05</v>
       </c>
       <c r="M39" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N39" s="6" t="n">
-        <v>3.17956475326815e-09</v>
+        <v>2.029133579003626e-07</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>3.17956475326815e-09</v>
+        <v>2.029133579003626e-07</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>1.591435246731849e-09</v>
+        <v>-2.029133579003626e-07</v>
       </c>
       <c r="Q39" s="6" t="n">
         <v>0</v>
@@ -3313,12 +3317,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>S15</t>
+          <t>S14</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Maple syrupUSDT (ERC-4626)</t>
+          <t>Maple syrupUSDC (ERC-4626)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3332,40 +3336,40 @@
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>0</v>
+        <v>1.176169e-06</v>
       </c>
       <c r="F40" s="6" t="n">
-        <v>0</v>
+        <v>1.18094e-06</v>
       </c>
       <c r="G40" s="6" t="n">
-        <v>0</v>
+        <v>4.771e-09</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>0</v>
+        <v>4.771e-09</v>
       </c>
       <c r="I40" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J40" s="6" t="n">
-        <v>0</v>
+        <v>4.771e-09</v>
       </c>
       <c r="K40" s="6" t="n">
         <v>0</v>
       </c>
       <c r="L40" s="6" t="n">
-        <v>0</v>
+        <v>1.176169e-06</v>
       </c>
       <c r="M40" s="7" t="n">
         <v>1</v>
       </c>
       <c r="N40" s="6" t="n">
-        <v>0</v>
+        <v>3.186545637782671e-09</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>0</v>
+        <v>3.186545637782671e-09</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>0</v>
+        <v>1.584454362217329e-09</v>
       </c>
       <c r="Q40" s="6" t="n">
         <v>0</v>
@@ -3378,12 +3382,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>S19</t>
+          <t>S15</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>BlackRock USD Institutional Digital Liquidity Fund (BUIDL-I)</t>
+          <t>Maple syrupUSDT (ERC-4626)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -3393,7 +3397,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E41" s="6" t="n">
@@ -3443,12 +3447,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>S20</t>
+          <t>S19</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Janus Henderson Anemoy Treasury Fund (JTRSY)</t>
+          <t>BlackRock USD Institutional Digital Liquidity Fund (BUIDL-I)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -3508,12 +3512,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>S21</t>
+          <t>S20</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Superstate Short Duration US Government Securities Fund (USTB)</t>
+          <t>Janus Henderson Anemoy Treasury Fund (JTRSY)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3551,7 +3555,7 @@
         <v>0</v>
       </c>
       <c r="M43" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N43" s="6" t="n">
         <v>0</v>
@@ -3568,21 +3572,17 @@
       <c r="R43" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S43" t="inlineStr">
-        <is>
-          <t>SDE (fixed)</t>
-        </is>
-      </c>
+      <c r="S43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>S22</t>
+          <t>S21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Superstate Crypto Carry Fund (USCC)</t>
+          <t>Superstate Short Duration US Government Securities Fund (USTB)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3620,7 +3620,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N44" s="6" t="n">
         <v>0</v>
@@ -3637,17 +3637,21 @@
       <c r="R44" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S44" t="inlineStr"/>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>SDE (fixed)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>S26</t>
+          <t>S22</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>USDC raw (ALM idle)</t>
+          <t>Superstate Crypto Carry Fund (USCC)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3657,7 +3661,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="E45" s="6" t="n">
@@ -3670,13 +3674,13 @@
         <v>0</v>
       </c>
       <c r="H45" s="6" t="n">
-        <v>8.562384e-08</v>
+        <v>0</v>
       </c>
       <c r="I45" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J45" s="6" t="n">
-        <v>8.562384e-08</v>
+        <v>0</v>
       </c>
       <c r="K45" s="6" t="n">
         <v>0</v>
@@ -3694,7 +3698,7 @@
         <v>0</v>
       </c>
       <c r="P45" s="6" t="n">
-        <v>8.562384e-08</v>
+        <v>0</v>
       </c>
       <c r="Q45" s="6" t="n">
         <v>0</v>
@@ -3707,12 +3711,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>S29</t>
+          <t>S26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>DAI raw (ALM idle)</t>
+          <t>USDC raw (ALM idle)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3735,13 +3739,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>0</v>
+        <v>8.562384e-08</v>
       </c>
       <c r="I46" s="6" t="n">
         <v>0</v>
       </c>
       <c r="J46" s="6" t="n">
-        <v>0</v>
+        <v>8.562384e-08</v>
       </c>
       <c r="K46" s="6" t="n">
         <v>0</v>
@@ -3759,7 +3763,7 @@
         <v>0</v>
       </c>
       <c r="P46" s="6" t="n">
-        <v>0</v>
+        <v>8.562384e-08</v>
       </c>
       <c r="Q46" s="6" t="n">
         <v>0</v>
@@ -3772,12 +3776,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>S31</t>
+          <t>S29</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
+          <t>DAI raw (ALM idle)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3815,7 +3819,7 @@
         <v>0</v>
       </c>
       <c r="M47" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N47" s="6" t="n">
         <v>0</v>
@@ -3832,31 +3836,27 @@
       <c r="R47" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S47" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>S37</t>
+          <t>S31</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Savings USDS / sUSDS proxy (Base — POL)</t>
+          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E48" s="6" t="n">
@@ -3884,7 +3884,7 @@
         <v>0</v>
       </c>
       <c r="M48" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N48" s="6" t="n">
         <v>0</v>
@@ -3901,17 +3901,21 @@
       <c r="R48" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S48" t="inlineStr"/>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>S38</t>
+          <t>S37</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>USDS raw (Base — POL)</t>
+          <t>Savings USDS / sUSDS proxy (Base — POL)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3921,7 +3925,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E49" s="6" t="n">
@@ -3949,7 +3953,7 @@
         <v>0</v>
       </c>
       <c r="M49" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N49" s="6" t="n">
         <v>0</v>
@@ -3966,31 +3970,27 @@
       <c r="R49" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S49" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>S42</t>
+          <t>S38</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Fluid Savings USDS (fsUSDS, Arbitrum)</t>
+          <t>USDS raw (Base — POL)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>arbitrum</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E50" s="6" t="n">
@@ -4018,7 +4018,7 @@
         <v>0</v>
       </c>
       <c r="M50" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N50" s="6" t="n">
         <v>0</v>
@@ -4035,17 +4035,21 @@
       <c r="R50" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S50" t="inlineStr"/>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>S44</t>
+          <t>S42</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>USDS raw (Arbitrum — POL)</t>
+          <t>Fluid Savings USDS (fsUSDS, Arbitrum)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -4055,14 +4059,14 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E51" s="6" t="n">
-        <v>90000000</v>
+        <v>0</v>
       </c>
       <c r="F51" s="6" t="n">
-        <v>90000000</v>
+        <v>0</v>
       </c>
       <c r="G51" s="6" t="n">
         <v>0</v>
@@ -4080,10 +4084,10 @@
         <v>0</v>
       </c>
       <c r="L51" s="6" t="n">
-        <v>90000000</v>
+        <v>0</v>
       </c>
       <c r="M51" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N51" s="6" t="n">
         <v>0</v>
@@ -4095,43 +4099,39 @@
         <v>0</v>
       </c>
       <c r="Q51" s="6" t="n">
-        <v>90000000</v>
+        <v>0</v>
       </c>
       <c r="R51" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S51" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>S47</t>
+          <t>S44</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Savings USDS / sUSDS proxy (Optimism — POL)</t>
+          <t>USDS raw (Arbitrum — POL)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>optimism</t>
+          <t>arbitrum</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E52" s="6" t="n">
-        <v>0</v>
+        <v>90000000</v>
       </c>
       <c r="F52" s="6" t="n">
-        <v>0</v>
+        <v>90000000</v>
       </c>
       <c r="G52" s="6" t="n">
         <v>0</v>
@@ -4149,10 +4149,10 @@
         <v>0</v>
       </c>
       <c r="L52" s="6" t="n">
-        <v>0</v>
+        <v>90000000</v>
       </c>
       <c r="M52" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N52" s="6" t="n">
         <v>0</v>
@@ -4164,22 +4164,26 @@
         <v>0</v>
       </c>
       <c r="Q52" s="6" t="n">
-        <v>0</v>
+        <v>90000000</v>
       </c>
       <c r="R52" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S52" t="inlineStr"/>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>S48</t>
+          <t>S47</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>USDS raw (Optimism — POL)</t>
+          <t>Savings USDS / sUSDS proxy (Optimism — POL)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -4189,7 +4193,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E53" s="6" t="n">
@@ -4217,7 +4221,7 @@
         <v>0</v>
       </c>
       <c r="M53" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N53" s="6" t="n">
         <v>0</v>
@@ -4234,31 +4238,27 @@
       <c r="R53" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S53" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>S51</t>
+          <t>S48</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Savings USDS / sUSDS proxy (Unichain — POL)</t>
+          <t>USDS raw (Optimism — POL)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>unichain</t>
+          <t>optimism</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E54" s="6" t="n">
@@ -4286,7 +4286,7 @@
         <v>0</v>
       </c>
       <c r="M54" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N54" s="6" t="n">
         <v>0</v>
@@ -4303,17 +4303,21 @@
       <c r="R54" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S54" t="inlineStr"/>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>S52</t>
+          <t>S51</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>USDS raw (Unichain — POL)</t>
+          <t>Savings USDS / sUSDS proxy (Unichain — POL)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -4323,7 +4327,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E55" s="6" t="n">
@@ -4351,7 +4355,7 @@
         <v>0</v>
       </c>
       <c r="M55" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N55" s="6" t="n">
         <v>0</v>
@@ -4368,21 +4372,17 @@
       <c r="R55" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S55" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>S53</t>
+          <t>S52</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>USDC raw (Unichain — ALM idle)</t>
+          <t>USDS raw (Unichain — POL)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -4420,7 +4420,7 @@
         <v>0</v>
       </c>
       <c r="M56" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N56" s="6" t="n">
         <v>0</v>
@@ -4437,22 +4437,26 @@
       <c r="R56" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="S56" t="inlineStr"/>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>S55</t>
+          <t>S53</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>USDC raw (Avalanche-C — ALM idle)</t>
+          <t>USDC raw (Unichain — ALM idle)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>avalanche_c</t>
+          <t>unichain</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -4507,140 +4511,177 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>S55</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>USDC raw (Avalanche-C — ALM idle)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>avalanche_c</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R58" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>PSM_CURVE_DEDUCT</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>PSM3 USDS + PSM3 USDC (SDE) + Curve idle USDS — BR deduction (unattributed)</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M58" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R58" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S58" t="inlineStr">
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M59" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R59" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S59" t="inlineStr">
         <is>
           <t>BR deduction from PSM3 USDS leg + PSM3 USDC leg (SDE, ≈$0 yield) + Curve idle USDS — not tracked per-venue; residual = sky_rev_br_reduction − Σ(known venue deduction_avg × effective_br_rate × n_days)</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>Position-only venues (PnL aggregated at prime level)</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>Venue</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Chain</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>Pricing cat.</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>Position SoM</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>Position EoM</t>
         </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>S56</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Spark Savings V2 — spUSDC vault</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>ethereum</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="E62" s="6" t="n">
-        <v>268629480.765079</v>
-      </c>
-      <c r="F62" s="6" t="n">
-        <v>309261582.801972</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>S57</t>
+          <t>S56</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Spark Savings V2 — spUSDT vault</t>
+          <t>Spark Savings V2 — spUSDC vault</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -4654,21 +4695,21 @@
         </is>
       </c>
       <c r="E63" s="6" t="n">
-        <v>404579096.135245</v>
+        <v>268629480.765079</v>
       </c>
       <c r="F63" s="6" t="n">
-        <v>367530003.125796</v>
+        <v>309261582.801972</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S59</t>
+          <t>S57</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Spark Savings V2 — spPYUSD vault</t>
+          <t>Spark Savings V2 — spUSDT vault</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -4682,26 +4723,26 @@
         </is>
       </c>
       <c r="E64" s="6" t="n">
-        <v>30570.4865</v>
+        <v>404579096.135245</v>
       </c>
       <c r="F64" s="6" t="n">
-        <v>230753.271254</v>
+        <v>367530003.125796</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>S60</t>
+          <t>S59</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Spark Savings V2 — spUSDC vault (Avalanche-C, CREATE2 same address)</t>
+          <t>Spark Savings V2 — spPYUSD vault</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>avalanche_c</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -4710,51 +4751,79 @@
         </is>
       </c>
       <c r="E65" s="6" t="n">
-        <v>12460370.146586</v>
+        <v>30570.4865</v>
       </c>
       <c r="F65" s="6" t="n">
-        <v>9475726.147763001</v>
+        <v>230753.271254</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>S60</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Spark Savings V2 — spUSDC vault (Avalanche-C, CREATE2 same address)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>avalanche_c</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="n">
+        <v>12460370.146586</v>
+      </c>
+      <c r="F66" s="6" t="n">
+        <v>9475726.147763001</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
           <t>S63</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>Spark Savings V2 — spUSDG vault (Robinhood Chain)</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>robinhood</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D67" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="E66" s="6" t="n">
+      <c r="E67" s="6" t="n">
         <v>21723212.723921</v>
       </c>
-      <c r="F66" s="6" t="n">
+      <c r="F67" s="6" t="n">
         <v>18807814.578688</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="inlineStr"/>
-      <c r="B67" s="5" t="inlineStr">
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" s="5" t="inlineStr">
         <is>
           <t>Aggregated actual_revenue (included in prime_agent_revenue, not in Venues body above)</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" s="9" t="n">
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4809,7 +4878,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>1967417205.777935</v>
+        <v>2026231562.920203</v>
       </c>
     </row>
     <row r="6">
@@ -4829,7 +4898,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>967417205.7779347</v>
+        <v>1026231562.920203</v>
       </c>
     </row>
     <row r="8">
@@ -4869,7 +4938,7 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>0.03655934922724602</v>
+        <v>0.03656182252293028</v>
       </c>
     </row>
     <row r="12">
@@ -4879,7 +4948,7 @@
         </is>
       </c>
       <c r="B12" s="11" t="n">
-        <v>-0.8520827266301976</v>
+        <v>-0.827349769787614</v>
       </c>
     </row>
     <row r="13">
@@ -4889,7 +4958,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>14237.93663854044</v>
+        <v>14237.93663854046</v>
       </c>
     </row>
     <row r="15">
@@ -4899,7 +4968,7 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>6123148.275689417</v>
+        <v>6306194.875294131</v>
       </c>
     </row>
     <row r="16">
@@ -4909,7 +4978,7 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>6108910.339050876</v>
+        <v>6291956.938655592</v>
       </c>
     </row>
     <row r="17">
@@ -4919,7 +4988,7 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>14237.93663854044</v>
+        <v>14237.93663854046</v>
       </c>
     </row>
     <row r="19">
@@ -4959,10 +5028,10 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>967417205.7779347</v>
+        <v>1026231562.920203</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>3010870.789395772</v>
+        <v>3193917.389000487</v>
       </c>
     </row>
     <row r="23">
@@ -4984,7 +5053,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>6084935.362245966</v>
+        <v>6267981.96185068</v>
       </c>
     </row>
     <row r="25">
@@ -4994,7 +5063,7 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>-7778.867166258307</v>
+        <v>-7825.937104839475</v>
       </c>
     </row>
     <row r="26">
@@ -5004,7 +5073,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>6077156.495079707</v>
+        <v>6260156.024745842</v>
       </c>
     </row>
     <row r="28">
@@ -5031,7 +5100,7 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>6084935.362245966</v>
+        <v>6267981.96185068</v>
       </c>
     </row>
     <row r="32">
@@ -5041,7 +5110,7 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>-2078993.144321223</v>
+        <v>-1895946.544716508</v>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
@@ -5171,7 +5240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5336,7 +5405,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>S61</t>
+          <t>S62</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5360,56 +5429,20 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Atlas — Uniswap Pools (designated 2026-05-26): "Investments by Spark in USDT in USDS/USDT Uniswap pools" — https://sky-atlas.io/#5f368e33-7a82-4244-a9ba-f285193ec043</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>PYUSD in PYUSD/USDS Uniswap V4</t>
+          <t>USDT in USDT/USDS Uniswap V4</t>
         </is>
       </c>
       <c r="I6" s="6" t="n">
-        <v>47.06993858116784</v>
+        <v>-7825.941992720887</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>47.06993858116784</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>S62</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>fixed</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2026-02-01</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>USDT in USDT/USDS Uniswap V4</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="n">
-        <v>-7825.941992720887</v>
-      </c>
-      <c r="J7" s="6" t="n">
         <v>-7825.941992720887</v>
       </c>
     </row>
@@ -5550,7 +5583,7 @@
         <v>10111001.62930237</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>118698545.210987</v>
+        <v>56003531.47877502</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>43456407.35738121</v>
@@ -5559,7 +5592,7 @@
         <v>390322896.0687824</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>1755866477.074628</v>
+        <v>1818561490.80684</v>
       </c>
       <c r="I6" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -5577,7 +5610,7 @@
         <v>0.03661299593747347</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>176195.5849832558</v>
+        <v>182489.9165878246</v>
       </c>
       <c r="O6" s="3" t="n">
         <v>241712.9264829505</v>
@@ -5599,7 +5632,7 @@
         <v>10100913.02149723</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>122814900.6419148</v>
+        <v>59737042.95218575</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>39340165.35218124</v>
@@ -5608,7 +5641,7 @@
         <v>380081346.7216024</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>1736824457.364285</v>
+        <v>1799902315.054014</v>
       </c>
       <c r="I7" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -5626,7 +5659,7 @@
         <v>0.03661299593747347</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>174283.8414594473</v>
+        <v>180616.6090843305</v>
       </c>
       <c r="O7" s="3" t="n">
         <v>238771.9704109938</v>
@@ -5648,7 +5681,7 @@
         <v>10096024.29960891</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>118803258.3720494</v>
+        <v>55902007.79758938</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>43345106.65294402</v>
@@ -5657,7 +5690,7 @@
         <v>380822312.0468913</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>1760617330.779413</v>
+        <v>1823518581.353873</v>
       </c>
       <c r="I8" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -5675,7 +5708,7 @@
         <v>0.03654216260414014</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>176478.4879926401</v>
+        <v>182793.5249611113</v>
       </c>
       <c r="O8" s="3" t="n">
         <v>241039.8433753375</v>
@@ -5697,7 +5730,7 @@
         <v>10111376.31186371</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>115834134.2645841</v>
+        <v>53138032.92749312</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>46322704.68907504</v>
@@ -5706,7 +5739,7 @@
         <v>377442762.5115625</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>1863125584.863853</v>
+        <v>1925821686.200944</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -5724,7 +5757,7 @@
         <v>0.03661299593747347</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>186963.975511396</v>
+        <v>193258.4163071964</v>
       </c>
       <c r="O9" s="3" t="n">
         <v>251188.4295072191</v>
@@ -5746,7 +5779,7 @@
         <v>10213659.95908268</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>121211032.7164317</v>
+        <v>57489610.06546267</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>40946104.38890742</v>
@@ -5755,7 +5788,7 @@
         <v>377118780.664318</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>1850028679.307531</v>
+        <v>1913750101.9585</v>
       </c>
       <c r="I10" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -5773,7 +5806,7 @@
         <v>0.0364713292708068</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>185260.9700993517</v>
+        <v>191658.3491029392</v>
       </c>
       <c r="O10" s="3" t="n">
         <v>249463.1964053061</v>
@@ -5795,7 +5828,7 @@
         <v>10222836.03395967</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>118536386.6105713</v>
+        <v>55697162.35399527</v>
       </c>
       <c r="F11" s="6" t="n">
         <v>43621876.13173749</v>
@@ -5804,7 +5837,7 @@
         <v>378324523.0900455</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>1845385333.735107</v>
+        <v>1908224557.991683</v>
       </c>
       <c r="I11" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -5822,7 +5855,7 @@
         <v>0.03654216260414014</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>184988.8604815783</v>
+        <v>191297.6702528653</v>
       </c>
       <c r="O11" s="3" t="n">
         <v>249313.1728130718</v>
@@ -5844,7 +5877,7 @@
         <v>10315500.32030975</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>109612940.5835957</v>
+        <v>47051142.91291972</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>52540305.80910107</v>
@@ -5853,7 +5886,7 @@
         <v>379064918.5542696</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>1847714176.967762</v>
+        <v>1910275974.638438</v>
       </c>
       <c r="I12" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -5871,7 +5904,7 @@
         <v>0.03632966260414013</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>184640.4753575982</v>
+        <v>190921.432596066</v>
       </c>
       <c r="O12" s="3" t="n">
         <v>249047.9199740752</v>
@@ -5893,7 +5926,7 @@
         <v>10312067.11217479</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>116780507.8168456</v>
+        <v>54131262.69424656</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>45375825.68351027</v>
@@ -5902,7 +5935,7 @@
         <v>379608384.4384824</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>1854293766.376791</v>
+        <v>1916943011.49939</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -5920,7 +5953,7 @@
         <v>0.03632966260414013</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>185301.0401313652</v>
+        <v>191590.776748409</v>
       </c>
       <c r="O13" s="3" t="n">
         <v>249763.0118276901</v>
@@ -5942,7 +5975,7 @@
         <v>10316900.39213798</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>116145591.4761823</v>
+        <v>53689767.45911231</v>
       </c>
       <c r="F14" s="6" t="n">
         <v>45997685.94893296</v>
@@ -5951,7 +5984,7 @@
         <v>376671380.9893584</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>1848629997.261933</v>
+        <v>1911085821.279003</v>
       </c>
       <c r="I14" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -5969,7 +6002,7 @@
         <v>0.03632966260414013</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>184732.4200957608</v>
+        <v>191002.7379982203</v>
       </c>
       <c r="O14" s="3" t="n">
         <v>248898.702716844</v>
@@ -5991,7 +6024,7 @@
         <v>10315368.28067446</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>119446433.3504283</v>
+        <v>56940396.60145326</v>
       </c>
       <c r="F15" s="6" t="n">
         <v>42700171.37311988</v>
@@ -6000,7 +6033,7 @@
         <v>368760529.6866171</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>1797504932.647244</v>
+        <v>1860010969.396219</v>
       </c>
       <c r="I15" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6018,7 +6051,7 @@
         <v>0.03640049593747347</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>179793.7295844561</v>
+        <v>186069.0886467554</v>
       </c>
       <c r="O15" s="3" t="n">
         <v>243165.974228541</v>
@@ -6040,7 +6073,7 @@
         <v>10312416.92489141</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>118645841.9705535</v>
+        <v>55797454.62041152</v>
       </c>
       <c r="F16" s="6" t="n">
         <v>43504485.64728707</v>
@@ -6049,7 +6082,7 @@
         <v>373262386.125073</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>1818675069.452996</v>
+        <v>1881523456.803138</v>
       </c>
       <c r="I16" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6067,7 +6100,7 @@
         <v>0.0364713292708068</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>182113.1915811483</v>
+        <v>188422.9212908163</v>
       </c>
       <c r="O16" s="3" t="n">
         <v>245937.4822794868</v>
@@ -6089,7 +6122,7 @@
         <v>10314003.14203688</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>123797953.747283</v>
+        <v>60625535.374295</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>38345804.82358488</v>
@@ -6098,7 +6131,7 @@
         <v>366534646.2498961</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>1871545578.210083</v>
+        <v>1934717996.583071</v>
       </c>
       <c r="I17" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6116,7 +6149,7 @@
         <v>0.03632966260414013</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>187033.0538593178</v>
+        <v>193375.3150030911</v>
       </c>
       <c r="O17" s="3" t="n">
         <v>250181.4058061647</v>
@@ -6138,7 +6171,7 @@
         <v>10314039.85394011</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>120305494.2332965</v>
+        <v>57503333.9399175</v>
       </c>
       <c r="F18" s="6" t="n">
         <v>41849956.0034882</v>
@@ -6147,7 +6180,7 @@
         <v>378300506.4139345</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>1871270048.554286</v>
+        <v>1934072208.847665</v>
       </c>
       <c r="I18" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6165,7 +6198,7 @@
         <v>0.03632966260414013</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>187005.3917707841</v>
+        <v>193310.480466645</v>
       </c>
       <c r="O18" s="3" t="n">
         <v>251336.1670615553</v>
@@ -6187,7 +6220,7 @@
         <v>10366023.19964889</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>121385124.1637922</v>
+        <v>58822846.50006123</v>
       </c>
       <c r="F19" s="6" t="n">
         <v>40766761.35986621</v>
@@ -6196,7 +6229,7 @@
         <v>398167107.6313812</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>1908261922.44069</v>
+        <v>1970824200.104421</v>
       </c>
       <c r="I19" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6214,7 +6247,7 @@
         <v>0.03632966260414013</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>190719.2297150573</v>
+        <v>197000.2351429309</v>
       </c>
       <c r="O19" s="3" t="n">
         <v>257049.3942935169</v>
@@ -6236,7 +6269,7 @@
         <v>10460758.25635528</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>122984092.0386592</v>
+        <v>60728568.70870018</v>
       </c>
       <c r="F20" s="6" t="n">
         <v>39168951.01282739</v>
@@ -6245,7 +6278,7 @@
         <v>411707743.9175714</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>1933862235.542659</v>
+        <v>1996117758.872618</v>
       </c>
       <c r="I20" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6263,7 +6296,7 @@
         <v>0.03632966260414013</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>193289.3999766485</v>
+        <v>199539.6084817214</v>
       </c>
       <c r="O20" s="3" t="n">
         <v>260988.6181614161</v>
@@ -6285,7 +6318,7 @@
         <v>10465932.21325058</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>123035635.4010988</v>
+        <v>60408955.44930481</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>39120098.62204416</v>
@@ -6294,7 +6327,7 @@
         <v>421609583.6052224</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>1959048560.027353</v>
+        <v>2021675239.979147</v>
       </c>
       <c r="I21" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6312,7 +6345,7 @@
         <v>0.03632966260414013</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>195818.007417171</v>
+        <v>202105.4785802448</v>
       </c>
       <c r="O21" s="3" t="n">
         <v>264512.1207817073</v>
@@ -6334,7 +6367,7 @@
         <v>10460616.09958957</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>113954568.7316583</v>
+        <v>56505129.66130627</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>48203049.61052532</v>
@@ -6343,7 +6376,7 @@
         <v>425134192.7347813</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>1930899662.518894</v>
+        <v>1988349101.589246</v>
       </c>
       <c r="I22" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6361,7 +6394,7 @@
         <v>0.03661299593747347</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>193768.2250610767</v>
+        <v>199535.9217003946</v>
       </c>
       <c r="O22" s="3" t="n">
         <v>262815.8507141541</v>
@@ -6383,7 +6416,7 @@
         <v>10464873.16045726</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>112431657.0870166</v>
+        <v>52351705.51743261</v>
       </c>
       <c r="F23" s="6" t="n">
         <v>49722766.02386782</v>
@@ -6392,7 +6425,7 @@
         <v>429236953.7797638</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>1937866048.939329</v>
+        <v>1997946000.508914</v>
       </c>
       <c r="I23" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6410,7 +6443,7 @@
         <v>0.03654216260414014</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>194273.5587992052</v>
+        <v>200305.3484975158</v>
       </c>
       <c r="O23" s="3" t="n">
         <v>263733.1920503536</v>
@@ -6432,7 +6465,7 @@
         <v>10470003.91638711</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>106532976.9280246</v>
+        <v>49480841.69692961</v>
       </c>
       <c r="F24" s="6" t="n">
         <v>55612983.26391467</v>
@@ -6441,7 +6474,7 @@
         <v>456649459.4870219</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>1986193874.771535</v>
+        <v>2043246010.00263</v>
       </c>
       <c r="I24" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6459,7 +6492,7 @@
         <v>0.03632966260414013</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>198543.2897377089</v>
+        <v>204271.098641732</v>
       </c>
       <c r="O24" s="3" t="n">
         <v>270754.6956901368</v>
@@ -6481,7 +6514,7 @@
         <v>10591383.26502531</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>94017998.83902577</v>
+        <v>41440417.79494276</v>
       </c>
       <c r="F25" s="6" t="n">
         <v>68132661.95247984</v>
@@ -6490,7 +6523,7 @@
         <v>460115553.4281456</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>1994871393.905399</v>
+        <v>2047448974.949482</v>
       </c>
       <c r="I25" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6508,7 +6541,7 @@
         <v>0.03640049593747347</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>199608.5422916562</v>
+        <v>204887.1236389877</v>
       </c>
       <c r="O25" s="3" t="n">
         <v>272180.5883061037</v>
@@ -6530,7 +6563,7 @@
         <v>10689446.68987206</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>106329945.9267851</v>
+        <v>40716605.36799709</v>
       </c>
       <c r="F26" s="6" t="n">
         <v>55802555.40412769</v>
@@ -6539,7 +6572,7 @@
         <v>427496697.7390748</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>1989386771.301211</v>
+        <v>2055000111.859999</v>
       </c>
       <c r="I26" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6557,7 +6590,7 @@
         <v>0.03654216260414014</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>199446.0357116074</v>
+        <v>206033.3557961762</v>
       </c>
       <c r="O26" s="3" t="n">
         <v>268751.2995686115</v>
@@ -6579,7 +6612,7 @@
         <v>10688408.27538944</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>103854611.8321672</v>
+        <v>40708384.96405221</v>
       </c>
       <c r="F27" s="6" t="n">
         <v>58299936.8409072</v>
@@ -6588,7 +6621,7 @@
         <v>414243116.5296448</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>2060955688.824644</v>
+        <v>2124101915.692759</v>
       </c>
       <c r="I27" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6606,7 +6639,7 @@
         <v>0.03654216260414014</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>206631.2721866586</v>
+        <v>212970.903806853</v>
       </c>
       <c r="O27" s="3" t="n">
         <v>274608.038082429</v>
@@ -6628,7 +6661,7 @@
         <v>10690988.55088899</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>100509176.2568168</v>
+        <v>36900147.82835181</v>
       </c>
       <c r="F28" s="6" t="n">
         <v>61650372.60727143</v>
@@ -6637,7 +6670,7 @@
         <v>428362900.2166361</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>2117100296.155342</v>
+        <v>2180709324.583807</v>
       </c>
       <c r="I28" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6655,7 +6688,7 @@
         <v>0.03654216260414014</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>212267.9688760822</v>
+        <v>218654.0639439184</v>
       </c>
       <c r="O28" s="3" t="n">
         <v>281663.0663007436</v>
@@ -6677,7 +6710,7 @@
         <v>10675390.01008535</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>100450167.6794079</v>
+        <v>39655786.88753793</v>
       </c>
       <c r="F29" s="6" t="n">
         <v>61708985.15202074</v>
@@ -6686,7 +6719,7 @@
         <v>400102506.1276009</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>2061819403.185396</v>
+        <v>2122613783.977266</v>
       </c>
       <c r="I29" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6704,7 +6737,7 @@
         <v>0.03654216260414014</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>206717.9856950314</v>
+        <v>212821.5012637959</v>
       </c>
       <c r="O29" s="3" t="n">
         <v>273274.2454478225</v>
@@ -6726,7 +6759,7 @@
         <v>10679624.19418858</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>96806566.86757933</v>
+        <v>38672566.79515033</v>
       </c>
       <c r="F30" s="6" t="n">
         <v>65323806.76275112</v>
@@ -6735,7 +6768,7 @@
         <v>401380571.2692359</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>2056487624.774785</v>
+        <v>2114621624.847214</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6753,7 +6786,7 @@
         <v>0.03661299593747347</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>206376.7601410284</v>
+        <v>212213.1839995321</v>
       </c>
       <c r="O30" s="3" t="n">
         <v>273058.8683603528</v>
@@ -6775,7 +6808,7 @@
         <v>10681637.27992404</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>94994247.49302587</v>
+        <v>36162849.01218788</v>
       </c>
       <c r="F31" s="6" t="n">
         <v>67165239.13105617</v>
@@ -6784,7 +6817,7 @@
         <v>410934023.6953909</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>2063619838.648978</v>
+        <v>2122451237.129816</v>
       </c>
       <c r="I31" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6802,7 +6835,7 @@
         <v>0.0364713292708068</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>206704.6783732144</v>
+        <v>212611.1182757654</v>
       </c>
       <c r="O31" s="3" t="n">
         <v>274349.0403957235</v>
@@ -6824,16 +6857,16 @@
         <v>10687300.73507782</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>89478570.4975764</v>
+        <v>32939858.6290874</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>72682306.08877099</v>
+        <v>87585552.09202559</v>
       </c>
       <c r="G32" s="6" t="n">
         <v>432413059.5419818</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>2153162366.536097</v>
+        <v>2194797832.401331</v>
       </c>
       <c r="I32" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6851,7 +6884,7 @@
         <v>0.0364713292708068</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>215694.3942960822</v>
+        <v>219874.4305232989</v>
       </c>
       <c r="O32" s="3" t="n">
         <v>285495.8747664904</v>
@@ -6873,16 +6906,16 @@
         <v>10702095.85803191</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>100167067.8351443</v>
+        <v>38890286.69818728</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>61984606.53330889</v>
+        <v>79077896.44486368</v>
       </c>
       <c r="G33" s="6" t="n">
         <v>385822680.9125517</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>2218633517.424233</v>
+        <v>2262817008.649635</v>
       </c>
       <c r="I33" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6900,7 +6933,7 @@
         <v>0.03654216260414014</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>222461.5030265996</v>
+        <v>226897.3509300406</v>
       </c>
       <c r="O33" s="3" t="n">
         <v>287586.0551159183</v>
@@ -6922,16 +6955,16 @@
         <v>10703038.74240102</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>97556631.18164769</v>
+        <v>36411873.27286968</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>64598585.3462756</v>
+        <v>89430518.4057503</v>
       </c>
       <c r="G34" s="6" t="n">
         <v>374700949.2558413</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>2289168923.271138</v>
+        <v>2325481748.120441</v>
       </c>
       <c r="I34" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6949,7 +6982,7 @@
         <v>0.03654216260414014</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>229542.9790138224</v>
+        <v>233188.6431184099</v>
       </c>
       <c r="O34" s="3" t="n">
         <v>293551.4034791795</v>
@@ -6971,16 +7004,16 @@
         <v>10702079.02186464</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>101135996.8440048</v>
+        <v>38268374.8890418</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>61022972.96983679</v>
+        <v>73934509.06061423</v>
       </c>
       <c r="G35" s="6" t="n">
         <v>374724871.851953</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>2295441223.813257</v>
+        <v>2345397309.677443</v>
       </c>
       <c r="I35" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -6998,7 +7031,7 @@
         <v>0.03654216260414014</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>230172.6931997742</v>
+        <v>235188.0867913373</v>
       </c>
       <c r="O35" s="3" t="n">
         <v>294183.7998621615</v>
@@ -7020,16 +7053,16 @@
         <v>10708476.71202994</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>103871515.4835148</v>
+        <v>42823370.20694085</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>58281574.25976945</v>
+        <v>69831218.80812408</v>
       </c>
       <c r="G36" s="6" t="n">
         <v>369328255.5143487</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>2311672594.439125</v>
+        <v>2361171095.167344</v>
       </c>
       <c r="I36" s="7" t="n">
         <v>0.03519999850777533</v>
@@ -7047,7 +7080,7 @@
         <v>0.03664455749990904</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>232082.7926243518</v>
+        <v>237052.2464766655</v>
       </c>
       <c r="O36" s="3" t="n">
         <v>295552.1523011315</v>
@@ -7072,7 +7105,7 @@
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" s="12" t="n">
-        <v>6108910.339050876</v>
+        <v>6291956.938655592</v>
       </c>
       <c r="O38" s="12" t="n">
         <v>8163928.506567189</v>

</xml_diff>